<commit_message>
feat(F-NAR-019): polish TREE-COL-003 et TREE-COL-027 xlsx
Alignement xlsx sur merged vocal après re-apply.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-003.xlsx
+++ b/stories/arbres/TREE-COL-003.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le tapis rouge, plié en boudin, roule hors des bras de papa. Il s'ouvre, chaud, avec une odeur de foin. Un grain de cerise glisse hors d'un pli. Le grain s'arrête, collé au bec de l'arrosoir. L'arrosoir vert est lourd, un peu bosselé. Le campement du cerisier sent la terre sèche. Maman pose la carafe, et un coussin rayé. Raphaël, l'eau, pour le pied de l'arbre. Le tapis est prêt, les genoux aussi. En ce moment, Raphaël saisit l'anse, trop vite. Je veux arroser, maintenant ! Mila arrive, les joues chaudes, les mains ouvertes. Je veux le tapis, pour raconter ! Les deux voix partent ensemble, trop fort. Papa tourne la carafe, il n'entend qu'un mélange. J'ai entendu un mélange. On n'a rien compris. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. La terre a soif ! Mila parle par-dessus, les mots se cognent. Personne ne se tourne. Le grain de cerise reste collé au bec, minuscule.</t>
+          <t>Le tapis rouge, plié en boudin, roule hors des bras de papa. Il s'ouvre, chaud, avec une odeur de foin. Un grain de cerise glisse hors d'un pli. Le grain s'arrête, collé au bec de l'arrosoir. L'arrosoir vert, lourd et bosselé, attend au campement du cerisier. Maman pose la carafe, et un coussin rayé. Raphaël, l'eau, pour le pied de l'arbre. Le tapis est prêt, les genoux aussi. En ce moment, Raphaël saisit l'anse, trop vite. Je veux arroser, maintenant ! Mila arrive, les joues chaudes, les mains ouvertes. Je veux le tapis, pour raconter ! Les deux voix partent ensemble, trop fort. Papa tourne la carafe, il n'entend qu'un mélange. J'ai entendu un mélange. On n'a rien compris. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. La terre a soif ! Mila parle par-dessus, les mots se cognent. Personne ne se tourne. Le grain de cerise reste collé au bec, minuscule.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le tapis rouge, plié en boudin, roule hors des bras de papa. Il s'ouvre, chaud, avec une odeur de foin. Un &lt;emphasis level="moderate"&gt;grain de cerise&lt;/emphasis&gt; glisse hors d'un pli. Le grain s'arrête, collé au bec de l'arrosoir. L'arrosoir vert est lourd, un peu bosselé. Le campement du cerisier sent la terre sèche. Maman pose la carafe, et un coussin rayé. Raphaël, l'eau, pour le pied de l'arbre. Le tapis est prêt, les genoux aussi. En ce moment, Raphaël saisit l'anse, trop vite. Je veux arroser, maintenant ! Mila arrive, les joues chaudes, les mains ouvertes. Je veux le tapis, pour raconter ! Les deux voix partent ensemble, trop fort. Papa tourne la carafe, il n'entend qu'un mélange. J'ai entendu un mélange. On n'a rien compris. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. La terre a soif ! Mila parle par-dessus, les mots se cognent. Personne ne se tourne. Le grain de cerise reste collé au bec, minuscule.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le tapis rouge, plié en boudin, roule hors des bras de papa. Il s'ouvre, chaud, avec une odeur de foin. Un &lt;emphasis level="moderate"&gt;grain de cerise&lt;/emphasis&gt; glisse hors d'un pli. Le grain s'arrête, collé au bec de l'arrosoir. L'arrosoir vert, lourd et bosselé, attend au campement du cerisier. Maman pose la carafe, et un coussin rayé. Raphaël, l'eau, pour le pied de l'arbre. Le tapis est prêt, les genoux aussi. En ce moment, Raphaël saisit l'anse, trop vite. Je veux arroser, maintenant ! Mila arrive, les joues chaudes, les mains ouvertes. Je veux le tapis, pour raconter ! Les deux voix partent ensemble, trop fort. Papa tourne la carafe, il n'entend qu'un mélange. J'ai entendu un mélange. On n'a rien compris. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. La terre a soif ! Mila parle par-dessus, les mots se cognent. Personne ne se tourne. Le grain de cerise reste collé au bec, minuscule.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le tapis rouge, plié en boudin, roule hors des bras de papa. Il s'ouvre, chaud, avec une odeur de foin. Un &lt;emphasis&gt;grain de cerise&lt;/emphasis&gt; glisse hors d'un pli. Le grain s'arrête, collé au bec de l'arrosoir. L'arrosoir vert est lourd, un peu bosselé. Le campement du cerisier sent la terre sèche. Maman pose la carafe, et un coussin rayé. Raphaël, l'eau, pour le pied de l'arbre. Le tapis est prêt, les genoux aussi. En ce moment, Raphaël saisit l'anse, trop vite. Je veux arroser, maintenant ! Mila arrive, les joues chaudes, les mains ouvertes. Je veux le tapis, pour raconter ! Les deux voix partent ensemble, trop fort. Papa tourne la carafe, il n'entend qu'un mélange. J'ai entendu un mélange. On n'a rien compris. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. La terre a soif ! Mila parle par-dessus, les mots se cognent. Personne ne se tourne. Le grain de cerise reste collé au bec, minuscule. [pause]</t>
+          <t>Le tapis rouge, plié en boudin, roule hors des bras de papa. Il s'ouvre, chaud, avec une odeur de foin. Un &lt;emphasis&gt;grain de cerise&lt;/emphasis&gt; glisse hors d'un pli. Le grain s'arrête, collé au bec de l'arrosoir. L'arrosoir vert, lourd et bosselé, attend au campement du cerisier. Maman pose la carafe, et un coussin rayé. Raphaël, l'eau, pour le pied de l'arbre. Le tapis est prêt, les genoux aussi. En ce moment, Raphaël saisit l'anse, trop vite. Je veux arroser, maintenant ! Mila arrive, les joues chaudes, les mains ouvertes. Je veux le tapis, pour raconter ! Les deux voix partent ensemble, trop fort. Papa tourne la carafe, il n'entend qu'un mélange. J'ai entendu un mélange. On n'a rien compris. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. La terre a soif ! Mila parle par-dessus, les mots se cognent. Personne ne se tourne. Le grain de cerise reste collé au bec, minuscule. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1345,8 +1345,7 @@
 narrateur|Il s'ouvre, chaud, avec une odeur de foin.
 narrateur|Un grain de cerise glisse hors d'un pli.
 narrateur|Le grain s'arrête, collé au bec de l'arrosoir.
-narrateur|L'arrosoir vert est lourd, un peu bosselé.
-narrateur|Le campement du cerisier sent la terre sèche.
+narrateur|L'arrosoir vert, lourd et bosselé, attend au campement du cerisier.
 narrateur|Maman pose la carafe, et un coussin rayé.
 papa|Raphaël, l'eau, pour le pied de l'arbre.
 maman|Le tapis est prêt, les genoux aussi.
@@ -17548,7 +17547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17605,6 +17604,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>